<commit_message>
fix: :bug: Memoria: correcciones v9 (correciones Alvaro)
</commit_message>
<xml_diff>
--- a/ceia-memoria/memoria/Tables/tablas-presentacion.xlsx
+++ b/ceia-memoria/memoria/Tables/tablas-presentacion.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documentos\Git Repositories\uba-ceia-memoria\ceia-memoria\memoria\Tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06497771-0852-4873-8692-FD98427D5142}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58CB0A2C-D671-4785-9689-F4955CC2D949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{5B0CB88E-CEC3-433C-A082-6CB6C22B5110}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{5B0CB88E-CEC3-433C-A082-6CB6C22B5110}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
     <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
     <sheet name="Hoja3" sheetId="3" r:id="rId3"/>
+    <sheet name="Hoja4" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="53">
   <si>
     <t>Autor y año</t>
   </si>
@@ -149,6 +150,54 @@
   </si>
   <si>
     <t>0,5</t>
+  </si>
+  <si>
+    <t>Local</t>
+  </si>
+  <si>
+    <t>GPU</t>
+  </si>
+  <si>
+    <t>NVIDIA GeForce RTX 4080 SUPER (16 GB GDDR6X)</t>
+  </si>
+  <si>
+    <t>Intel Core i7-12700KF (12 núcleos)</t>
+  </si>
+  <si>
+    <t>128 GB DDR5 (5600 MHz)</t>
+  </si>
+  <si>
+    <t>1 TB NVMe</t>
+  </si>
+  <si>
+    <t>Windows 11</t>
+  </si>
+  <si>
+    <t>NVIDIA A100 (80 GB HBM2e)</t>
+  </si>
+  <si>
+    <t>Intel(R) Xeon(R) CPU @ 2,20 GHz (12 núcleos)</t>
+  </si>
+  <si>
+    <t>167 GB</t>
+  </si>
+  <si>
+    <t>Ubuntu 24.04</t>
+  </si>
+  <si>
+    <t>CPU</t>
+  </si>
+  <si>
+    <t>RAM</t>
+  </si>
+  <si>
+    <t>Storage</t>
+  </si>
+  <si>
+    <t>SO</t>
+  </si>
+  <si>
+    <t>Item</t>
   </si>
 </sst>
 </file>
@@ -287,6 +336,18 @@
     <tableColumn id="1" xr3:uid="{9E3652E4-D8EB-4407-B2BD-F75E55006027}" name="Fase"/>
     <tableColumn id="2" xr3:uid="{933AD82A-187A-4D57-96D0-A754C7648C2B}" name="Técnica"/>
     <tableColumn id="3" xr3:uid="{34E52501-6556-4935-B144-4A279D2AFB62}" name="Thresshold"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{D0570CEA-BB31-49AD-B5FC-0C510495F2C4}" name="Tabla5" displayName="Tabla5" ref="A1:C6" totalsRowShown="0">
+  <autoFilter ref="A1:C6" xr:uid="{D0570CEA-BB31-49AD-B5FC-0C510495F2C4}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{6CF44246-5875-42B0-9EA4-5979E4A8FA36}" name="Item"/>
+    <tableColumn id="2" xr3:uid="{E58E233F-7C34-4C0A-BCC1-A434727ADB5C}" name="Local"/>
+    <tableColumn id="3" xr3:uid="{7F6E8ADA-F441-414F-81BA-8230DEA65FBB}" name="Nube"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -819,4 +880,89 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05F44C0D-02B9-4B74-B0F6-FEA6C6AF8CF3}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="44" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>